<commit_message>
Add all process.xaml activities
</commit_message>
<xml_diff>
--- a/Data/Clients.xlsx
+++ b/Data/Clients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://roboyo-my.sharepoint.com/personal/adelina_mancilla_roboyo_mx/Documents/Documents/UiPath/RoboticEnterpriseFrameworkPractice/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E378C00B-F72F-4F14-87B5-27767988796B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{E378C00B-F72F-4F14-87B5-27767988796B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16FB1E73-B5C0-41D9-AED4-BD81442C0E55}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="10584" windowWidth="23256" windowHeight="12456" xr2:uid="{7F8C78F4-37F2-4E28-BC2A-47EBBEAF3486}"/>
+    <workbookView xWindow="-19992" yWindow="14772" windowWidth="14376" windowHeight="8160" xr2:uid="{7F8C78F4-37F2-4E28-BC2A-47EBBEAF3486}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Name</t>
   </si>
   <si>
-    <t>First Name</t>
-  </si>
-  <si>
     <t>Secound Name</t>
   </si>
   <si>
@@ -53,9 +50,6 @@
     <t>Date</t>
   </si>
   <si>
-    <t>mariana.lopez@yahoo.com</t>
-  </si>
-  <si>
     <t>Mariana</t>
   </si>
   <si>
@@ -86,15 +80,9 @@
     <t>maguilarrios25@gmail.com</t>
   </si>
   <si>
-    <t>29/06/2025</t>
-  </si>
-  <si>
     <t>diego.ramirez@gmail.com</t>
   </si>
   <si>
-    <t>30/06/2025</t>
-  </si>
-  <si>
     <t>fer.ruizgomez@yahoo.com</t>
   </si>
   <si>
@@ -107,9 +95,6 @@
     <t>lftorres2025@gmail.com</t>
   </si>
   <si>
-    <t>regina.morales@yahoo.com</t>
-  </si>
-  <si>
     <t>eduardo.jp@gmail.com</t>
   </si>
   <si>
@@ -119,24 +104,9 @@
     <t>Sofia</t>
   </si>
   <si>
-    <t xml:space="preserve"> Hernández</t>
-  </si>
-  <si>
     <t xml:space="preserve"> López </t>
   </si>
   <si>
-    <t xml:space="preserve"> Gómez</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Mendoza</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Paredes</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Ríos</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
@@ -168,6 +138,30 @@
   </si>
   <si>
     <t>Fernadez</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Paredes</t>
+  </si>
+  <si>
+    <t>Mendoza</t>
+  </si>
+  <si>
+    <t>Hernández</t>
+  </si>
+  <si>
+    <t>Gómez</t>
+  </si>
+  <si>
+    <t>Ríos</t>
+  </si>
+  <si>
+    <t>mariana.lopez@gmail.com</t>
+  </si>
+  <si>
+    <t>regina.morales@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -257,7 +251,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -280,6 +274,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -296,6 +291,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -629,182 +628,182 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>16</v>
+        <v>40</v>
+      </c>
+      <c r="E2" s="10">
+        <v>45838</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
+      </c>
+      <c r="E3" s="10">
+        <v>45839</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="E4" s="10">
+        <v>45840</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="1" t="s">
         <v>16</v>
+      </c>
+      <c r="E5" s="10">
+        <v>45841</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="E6" s="10">
+        <v>45842</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="E7" s="10">
+        <v>45843</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>18</v>
+        <v>41</v>
+      </c>
+      <c r="E8" s="10">
+        <v>45844</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>31</v>
-      </c>
       <c r="D9" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
+      </c>
+      <c r="E9" s="10">
+        <v>45845</v>
       </c>
       <c r="N9" s="3"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="E10" s="10">
+        <v>45846</v>
       </c>
       <c r="N10" s="2"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
+      </c>
+      <c r="E11" s="10">
+        <v>45847</v>
       </c>
       <c r="N11" s="2"/>
     </row>
@@ -839,16 +838,16 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" display="mailto:mariana.lopez@yahoo.com" xr:uid="{1EBA8DD9-F8A0-4A03-AE7E-6666EF1E334E}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{1EBA8DD9-F8A0-4A03-AE7E-6666EF1E334E}"/>
     <hyperlink ref="D3" r:id="rId2" display="mailto:diego.ramirez@gmail.com" xr:uid="{0BED1E9E-3CA2-4A04-9909-AE505C48AB93}"/>
     <hyperlink ref="D4" r:id="rId3" display="mailto:fer.ruizgomez@yahoo.com" xr:uid="{02E5AC7F-F914-4559-920B-5C93F1DE025D}"/>
     <hyperlink ref="D5" r:id="rId4" display="mailto:carlos.sanchez25@gmail.com" xr:uid="{B45435C6-84CA-4A92-ACE6-E03C64BA7128}"/>
     <hyperlink ref="D6" r:id="rId5" display="mailto:alejandra.ortega@yahoo.com" xr:uid="{C6589B32-97CB-4466-A782-4D9F25974975}"/>
     <hyperlink ref="D7" r:id="rId6" display="mailto:lftorres2025@gmail.com" xr:uid="{8FB94BF2-E957-4ED8-9C56-28E09E3DEF7B}"/>
-    <hyperlink ref="D8" r:id="rId7" display="mailto:regina.morales@yahoo.com" xr:uid="{F4C70AC8-76CC-421E-8A36-935AD38C7AEB}"/>
-    <hyperlink ref="D9" r:id="rId8" display="mailto:eduardo.jp@gmail.com" xr:uid="{AD3A7C35-D535-4F85-A2F8-E0E3724BA099}"/>
-    <hyperlink ref="D10" r:id="rId9" display="mailto:sofia.castillo93@yahoo.com" xr:uid="{0F918A23-29DE-4FD3-A0CE-B4AFFC16A4CA}"/>
-    <hyperlink ref="D11" r:id="rId10" display="mailto:maguilarrios25@gmail.com" xr:uid="{AF802068-803C-43E2-A1DB-649B0C358321}"/>
+    <hyperlink ref="D9" r:id="rId7" display="mailto:eduardo.jp@gmail.com" xr:uid="{AD3A7C35-D535-4F85-A2F8-E0E3724BA099}"/>
+    <hyperlink ref="D10" r:id="rId8" display="mailto:sofia.castillo93@yahoo.com" xr:uid="{0F918A23-29DE-4FD3-A0CE-B4AFFC16A4CA}"/>
+    <hyperlink ref="D11" r:id="rId9" display="mailto:maguilarrios25@gmail.com" xr:uid="{AF802068-803C-43E2-A1DB-649B0C358321}"/>
+    <hyperlink ref="D8" r:id="rId10" xr:uid="{F4C70AC8-76CC-421E-8A36-935AD38C7AEB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Notas a mejorar parte 1
</commit_message>
<xml_diff>
--- a/Data/Clients.xlsx
+++ b/Data/Clients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://roboyo-my.sharepoint.com/personal/adelina_mancilla_roboyo_mx/Documents/Documents/UiPath/RoboticEnterpriseFrameworkPractice/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{E378C00B-F72F-4F14-87B5-27767988796B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16FB1E73-B5C0-41D9-AED4-BD81442C0E55}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{E378C00B-F72F-4F14-87B5-27767988796B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{555E36CE-E0D7-40D0-84EA-56631856350E}"/>
   <bookViews>
-    <workbookView xWindow="-19992" yWindow="14772" windowWidth="14376" windowHeight="8160" xr2:uid="{7F8C78F4-37F2-4E28-BC2A-47EBBEAF3486}"/>
+    <workbookView xWindow="-23148" yWindow="10584" windowWidth="23256" windowHeight="12456" xr2:uid="{7F8C78F4-37F2-4E28-BC2A-47EBBEAF3486}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Name</t>
   </si>
@@ -104,12 +104,6 @@
     <t>Sofia</t>
   </si>
   <si>
-    <t xml:space="preserve"> López </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>Torres</t>
   </si>
   <si>
@@ -162,6 +156,15 @@
   </si>
   <si>
     <t>regina.morales@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">López </t>
+  </si>
+  <si>
+    <t>Alvarez</t>
+  </si>
+  <si>
+    <t>Juarez</t>
   </si>
 </sst>
 </file>
@@ -291,10 +294,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -628,7 +627,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -645,13 +644,13 @@
         <v>4</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E2" s="10">
         <v>45838</v>
@@ -662,7 +661,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="5" t="s">
@@ -677,10 +676,10 @@
         <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>15</v>
@@ -694,9 +693,11 @@
         <v>7</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="4"/>
+        <v>26</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
@@ -709,10 +710,10 @@
         <v>8</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>17</v>
@@ -726,10 +727,10 @@
         <v>9</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>18</v>
@@ -743,13 +744,13 @@
         <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E8" s="10">
         <v>45844</v>
@@ -760,10 +761,10 @@
         <v>11</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>19</v>
@@ -778,7 +779,7 @@
         <v>21</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="5" t="s">
@@ -794,10 +795,10 @@
         <v>12</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>13</v>
@@ -845,7 +846,7 @@
     <hyperlink ref="D6" r:id="rId5" display="mailto:alejandra.ortega@yahoo.com" xr:uid="{C6589B32-97CB-4466-A782-4D9F25974975}"/>
     <hyperlink ref="D7" r:id="rId6" display="mailto:lftorres2025@gmail.com" xr:uid="{8FB94BF2-E957-4ED8-9C56-28E09E3DEF7B}"/>
     <hyperlink ref="D9" r:id="rId7" display="mailto:eduardo.jp@gmail.com" xr:uid="{AD3A7C35-D535-4F85-A2F8-E0E3724BA099}"/>
-    <hyperlink ref="D10" r:id="rId8" display="mailto:sofia.castillo93@yahoo.com" xr:uid="{0F918A23-29DE-4FD3-A0CE-B4AFFC16A4CA}"/>
+    <hyperlink ref="D10" r:id="rId8" xr:uid="{0F918A23-29DE-4FD3-A0CE-B4AFFC16A4CA}"/>
     <hyperlink ref="D11" r:id="rId9" display="mailto:maguilarrios25@gmail.com" xr:uid="{AF802068-803C-43E2-A1DB-649B0C358321}"/>
     <hyperlink ref="D8" r:id="rId10" xr:uid="{F4C70AC8-76CC-421E-8A36-935AD38C7AEB}"/>
   </hyperlinks>

</xml_diff>